<commit_message>
Full backup 03/06/2026 13:56:55
</commit_message>
<xml_diff>
--- a/Tubex_v10_29.xlsx
+++ b/Tubex_v10_29.xlsx
@@ -832,7 +832,7 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="21"/>
     <xf numFmtId="43" fontId="24" fillId="0" borderId="21"/>
   </cellStyleXfs>
-  <cellXfs count="289">
+  <cellXfs count="295">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1582,6 +1582,24 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="50" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="48" fillId="12" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="12" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="49" fillId="12" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="13" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="13" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="49" fillId="13" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -49134,31 +49152,31 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="246">
-      <c r="A4" s="263" t="n">
+      <c r="A4" s="289" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="263" t="n">
+      <c r="B4" s="289" t="n">
         <v>8001</v>
       </c>
-      <c r="C4" s="264" t="inlineStr">
+      <c r="C4" s="290" t="inlineStr">
         <is>
           <t>Alpha Labs PVT LTD</t>
         </is>
       </c>
-      <c r="D4" s="264" t="inlineStr">
+      <c r="D4" s="290" t="inlineStr">
         <is>
           <t>TRANSPARENT BOTTLE 150ML</t>
         </is>
       </c>
-      <c r="E4" s="263" t="inlineStr">
+      <c r="E4" s="289" t="inlineStr">
         <is>
           <t>150ml</t>
         </is>
       </c>
-      <c r="F4" s="265" t="n">
+      <c r="F4" s="291" t="n">
         <v>33465</v>
       </c>
-      <c r="G4" s="263" t="inlineStr">
+      <c r="G4" s="289" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -49174,31 +49192,31 @@
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="246">
-      <c r="A5" s="263" t="n">
+      <c r="A5" s="289" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="263" t="n">
+      <c r="B5" s="289" t="n">
         <v>3726</v>
       </c>
-      <c r="C5" s="264" t="inlineStr">
+      <c r="C5" s="290" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D5" s="264" t="inlineStr">
+      <c r="D5" s="290" t="inlineStr">
         <is>
           <t>TUBES</t>
         </is>
       </c>
-      <c r="E5" s="263" t="inlineStr">
+      <c r="E5" s="289" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="F5" s="265" t="n">
+      <c r="F5" s="291" t="n">
         <v>22512</v>
       </c>
-      <c r="G5" s="263" t="inlineStr">
+      <c r="G5" s="289" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -49214,31 +49232,31 @@
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="246">
-      <c r="A6" s="263" t="n">
+      <c r="A6" s="289" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="263" t="n">
+      <c r="B6" s="289" t="n">
         <v>3447</v>
       </c>
-      <c r="C6" s="264" t="inlineStr">
+      <c r="C6" s="290" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D6" s="264" t="inlineStr">
+      <c r="D6" s="290" t="inlineStr">
         <is>
           <t>S 43 25MM</t>
         </is>
       </c>
-      <c r="E6" s="263" t="inlineStr">
+      <c r="E6" s="289" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="F6" s="265" t="n">
+      <c r="F6" s="291" t="n">
         <v>89000</v>
       </c>
-      <c r="G6" s="263" t="inlineStr">
+      <c r="G6" s="289" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -49254,31 +49272,31 @@
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="246">
-      <c r="A7" s="263" t="n">
+      <c r="A7" s="289" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="263" t="n">
+      <c r="B7" s="289" t="n">
         <v>4050</v>
       </c>
-      <c r="C7" s="264" t="inlineStr">
+      <c r="C7" s="290" t="inlineStr">
         <is>
           <t>Professional Beauty Solution (PVT) LTD.Pakistan</t>
         </is>
       </c>
-      <c r="D7" s="264" t="inlineStr">
+      <c r="D7" s="290" t="inlineStr">
         <is>
           <t>EAZICOLOR PREMIUM HAIR COLOUR 60ML</t>
         </is>
       </c>
-      <c r="E7" s="263" t="inlineStr">
+      <c r="E7" s="289" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F7" s="265" t="n">
+      <c r="F7" s="291" t="n">
         <v>9450</v>
       </c>
-      <c r="G7" s="263" t="inlineStr">
+      <c r="G7" s="289" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -49294,31 +49312,31 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="246">
-      <c r="A8" s="263" t="n">
+      <c r="A8" s="289" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="263" t="n">
+      <c r="B8" s="289" t="n">
         <v>6337</v>
       </c>
-      <c r="C8" s="264" t="inlineStr">
+      <c r="C8" s="290" t="inlineStr">
         <is>
           <t>Al-Rehman Group</t>
         </is>
       </c>
-      <c r="D8" s="264" t="inlineStr">
+      <c r="D8" s="290" t="inlineStr">
         <is>
           <t>ACTIVE PRO HAIR COLOR CREAM 60ML</t>
         </is>
       </c>
-      <c r="E8" s="263" t="inlineStr">
+      <c r="E8" s="289" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F8" s="265" t="n">
+      <c r="F8" s="291" t="n">
         <v>15680</v>
       </c>
-      <c r="G8" s="263" t="inlineStr">
+      <c r="G8" s="289" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -49334,31 +49352,31 @@
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="246">
-      <c r="A9" s="263" t="n">
+      <c r="A9" s="289" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="263" t="n">
+      <c r="B9" s="289" t="n">
         <v>6416</v>
       </c>
-      <c r="C9" s="264" t="inlineStr">
+      <c r="C9" s="290" t="inlineStr">
         <is>
           <t>Al-Rehman Group</t>
         </is>
       </c>
-      <c r="D9" s="264" t="inlineStr">
+      <c r="D9" s="290" t="inlineStr">
         <is>
           <t>SIGNATURE HAIR COLOR CREAM 60ML</t>
         </is>
       </c>
-      <c r="E9" s="263" t="inlineStr">
+      <c r="E9" s="289" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F9" s="265" t="n">
+      <c r="F9" s="291" t="n">
         <v>15435</v>
       </c>
-      <c r="G9" s="263" t="inlineStr">
+      <c r="G9" s="289" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -49374,31 +49392,31 @@
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="246">
-      <c r="A10" s="263" t="n">
+      <c r="A10" s="289" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="263" t="n">
+      <c r="B10" s="289" t="n">
         <v>5782</v>
       </c>
-      <c r="C10" s="264" t="inlineStr">
+      <c r="C10" s="290" t="inlineStr">
         <is>
           <t>Mega Grey</t>
         </is>
       </c>
-      <c r="D10" s="264" t="inlineStr">
+      <c r="D10" s="290" t="inlineStr">
         <is>
           <t>M.G</t>
         </is>
       </c>
-      <c r="E10" s="263" t="inlineStr">
+      <c r="E10" s="289" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="F10" s="265" t="n">
+      <c r="F10" s="291" t="n">
         <v>63648</v>
       </c>
-      <c r="G10" s="263" t="inlineStr">
+      <c r="G10" s="289" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -49414,31 +49432,31 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="246">
-      <c r="A11" s="263" t="n">
+      <c r="A11" s="289" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="263" t="n">
+      <c r="B11" s="289" t="n">
         <v>6531</v>
       </c>
-      <c r="C11" s="264" t="inlineStr">
+      <c r="C11" s="290" t="inlineStr">
         <is>
           <t>Adore</t>
         </is>
       </c>
-      <c r="D11" s="264" t="inlineStr">
+      <c r="D11" s="290" t="inlineStr">
         <is>
           <t>V-HC BLACK</t>
         </is>
       </c>
-      <c r="E11" s="263" t="inlineStr">
+      <c r="E11" s="289" t="inlineStr">
         <is>
           <t>35</t>
         </is>
       </c>
-      <c r="F11" s="265" t="n">
+      <c r="F11" s="291" t="n">
         <v>4380</v>
       </c>
-      <c r="G11" s="263" t="inlineStr">
+      <c r="G11" s="289" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -49454,31 +49472,31 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="246">
-      <c r="A12" s="267" t="n">
+      <c r="A12" s="292" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="267" t="n">
+      <c r="B12" s="292" t="n">
         <v>6515</v>
       </c>
-      <c r="C12" s="268" t="inlineStr">
+      <c r="C12" s="293" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D12" s="268" t="inlineStr">
+      <c r="D12" s="293" t="inlineStr">
         <is>
           <t>H.H 100GM</t>
         </is>
       </c>
-      <c r="E12" s="267" t="inlineStr">
+      <c r="E12" s="292" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="F12" s="269" t="n">
+      <c r="F12" s="294" t="n">
         <v>38896</v>
       </c>
-      <c r="G12" s="267" t="inlineStr">
+      <c r="G12" s="292" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -49494,31 +49512,31 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="246">
-      <c r="A13" s="267" t="n">
+      <c r="A13" s="292" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="267" t="n">
+      <c r="B13" s="292" t="n">
         <v>6530</v>
       </c>
-      <c r="C13" s="268" t="inlineStr">
+      <c r="C13" s="293" t="inlineStr">
         <is>
           <t>Adore</t>
         </is>
       </c>
-      <c r="D13" s="268" t="inlineStr">
+      <c r="D13" s="293" t="inlineStr">
         <is>
           <t>V- HC BROWN</t>
         </is>
       </c>
-      <c r="E13" s="267" t="inlineStr">
+      <c r="E13" s="292" t="inlineStr">
         <is>
           <t>35</t>
         </is>
       </c>
-      <c r="F13" s="269" t="n">
+      <c r="F13" s="294" t="n">
         <v>15000</v>
       </c>
-      <c r="G13" s="267" t="inlineStr">
+      <c r="G13" s="292" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -49534,31 +49552,31 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="246">
-      <c r="A14" s="267" t="n">
+      <c r="A14" s="292" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="267" t="n">
+      <c r="B14" s="292" t="n">
         <v>6206</v>
       </c>
-      <c r="C14" s="268" t="inlineStr">
+      <c r="C14" s="293" t="inlineStr">
         <is>
           <t>Golden Pearl Cosmetics (PVT) LTD</t>
         </is>
       </c>
-      <c r="D14" s="268" t="inlineStr">
+      <c r="D14" s="293" t="inlineStr">
         <is>
           <t>HELLO HAIR COLOR</t>
         </is>
       </c>
-      <c r="E14" s="267" t="inlineStr">
+      <c r="E14" s="292" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F14" s="269" t="n">
+      <c r="F14" s="294" t="n">
         <v>98674</v>
       </c>
-      <c r="G14" s="267" t="inlineStr">
+      <c r="G14" s="292" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -49574,31 +49592,31 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="246">
-      <c r="A15" s="267" t="n">
+      <c r="A15" s="292" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="267" t="n">
+      <c r="B15" s="292" t="n">
         <v>3726</v>
       </c>
-      <c r="C15" s="268" t="inlineStr">
+      <c r="C15" s="293" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D15" s="268" t="inlineStr">
+      <c r="D15" s="293" t="inlineStr">
         <is>
           <t>TUBES</t>
         </is>
       </c>
-      <c r="E15" s="267" t="inlineStr">
+      <c r="E15" s="292" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="F15" s="269" t="n">
+      <c r="F15" s="294" t="n">
         <v>9744</v>
       </c>
-      <c r="G15" s="267" t="inlineStr">
+      <c r="G15" s="292" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -49614,31 +49632,31 @@
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="246">
-      <c r="A16" s="267" t="n">
+      <c r="A16" s="292" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="267" t="n">
+      <c r="B16" s="292" t="n">
         <v>5782</v>
       </c>
-      <c r="C16" s="268" t="inlineStr">
+      <c r="C16" s="293" t="inlineStr">
         <is>
           <t>Mega Grey</t>
         </is>
       </c>
-      <c r="D16" s="268" t="inlineStr">
+      <c r="D16" s="293" t="inlineStr">
         <is>
           <t>M.G</t>
         </is>
       </c>
-      <c r="E16" s="267" t="inlineStr">
+      <c r="E16" s="292" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="F16" s="269" t="n">
+      <c r="F16" s="294" t="n">
         <v>10500</v>
       </c>
-      <c r="G16" s="267" t="inlineStr">
+      <c r="G16" s="292" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -49654,31 +49672,31 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="246">
-      <c r="A17" s="267" t="n">
+      <c r="A17" s="292" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="267" t="n">
+      <c r="B17" s="292" t="n">
         <v>6624</v>
       </c>
-      <c r="C17" s="268" t="inlineStr">
+      <c r="C17" s="293" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D17" s="268" t="inlineStr">
+      <c r="D17" s="293" t="inlineStr">
         <is>
           <t>S-45 DIA 19MM</t>
         </is>
       </c>
-      <c r="E17" s="267" t="inlineStr">
+      <c r="E17" s="292" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="F17" s="269" t="n">
+      <c r="F17" s="294" t="n">
         <v>15288</v>
       </c>
-      <c r="G17" s="267" t="inlineStr">
+      <c r="G17" s="292" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -49694,31 +49712,31 @@
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="246">
-      <c r="A18" s="267" t="n">
+      <c r="A18" s="292" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="267" t="n">
+      <c r="B18" s="292" t="n">
         <v>5699</v>
       </c>
-      <c r="C18" s="268" t="inlineStr">
+      <c r="C18" s="293" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D18" s="268" t="inlineStr">
+      <c r="D18" s="293" t="inlineStr">
         <is>
           <t>S-43 DIA 20.5</t>
         </is>
       </c>
-      <c r="E18" s="267" t="inlineStr">
+      <c r="E18" s="292" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F18" s="269" t="n">
+      <c r="F18" s="294" t="n">
         <v>13770</v>
       </c>
-      <c r="G18" s="267" t="inlineStr">
+      <c r="G18" s="292" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -49734,31 +49752,31 @@
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="246">
-      <c r="A19" s="267" t="n">
+      <c r="A19" s="292" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="267" t="n">
+      <c r="B19" s="292" t="n">
         <v>5731</v>
       </c>
-      <c r="C19" s="268" t="inlineStr">
+      <c r="C19" s="293" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D19" s="268" t="inlineStr">
+      <c r="D19" s="293" t="inlineStr">
         <is>
           <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
         </is>
       </c>
-      <c r="E19" s="267" t="inlineStr">
+      <c r="E19" s="292" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F19" s="269" t="n">
+      <c r="F19" s="294" t="n">
         <v>51000</v>
       </c>
-      <c r="G19" s="267" t="inlineStr">
+      <c r="G19" s="292" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>

</xml_diff>

<commit_message>
Full backup 03/06/2026 14:00:16
</commit_message>
<xml_diff>
--- a/Tubex_v10_29.xlsx
+++ b/Tubex_v10_29.xlsx
@@ -832,7 +832,7 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="21"/>
     <xf numFmtId="43" fontId="24" fillId="0" borderId="21"/>
   </cellStyleXfs>
-  <cellXfs count="295">
+  <cellXfs count="301">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1600,6 +1600,24 @@
     <xf numFmtId="3" fontId="49" fillId="13" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="48" fillId="12" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="12" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="49" fillId="12" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="13" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="13" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="49" fillId="13" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -40767,172 +40785,398 @@
       <c r="S10" s="259" t="n"/>
     </row>
     <row r="11" hidden="1" ht="15" customHeight="1" s="246">
-      <c r="A11" s="193" t="n"/>
-      <c r="B11" s="194" t="n"/>
-      <c r="C11" s="194" t="n"/>
-      <c r="D11" s="194" t="n"/>
-      <c r="E11" s="194" t="n"/>
-      <c r="F11" s="194" t="n"/>
-      <c r="G11" s="195" t="n"/>
-      <c r="H11" s="195" t="n"/>
-      <c r="I11" s="195" t="n"/>
-      <c r="J11" s="196" t="n"/>
-      <c r="K11" s="194" t="n"/>
-      <c r="L11" s="194" t="n"/>
-      <c r="M11" s="194" t="n"/>
-      <c r="N11" s="194" t="n"/>
-      <c r="O11" s="194" t="n"/>
-      <c r="P11" s="194" t="n"/>
-      <c r="Q11" s="194" t="n"/>
-      <c r="R11" s="194" t="n"/>
-      <c r="S11" s="194" t="n"/>
+      <c r="A11" s="262" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B11" s="259" t="inlineStr">
+        <is>
+          <t>Lacquer-02</t>
+        </is>
+      </c>
+      <c r="C11" s="259" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D11" s="259" t="inlineStr">
+        <is>
+          <t>TUBES</t>
+        </is>
+      </c>
+      <c r="E11" s="259" t="n">
+        <v>25</v>
+      </c>
+      <c r="F11" s="259" t="n">
+        <v>3726</v>
+      </c>
+      <c r="G11" s="260" t="n">
+        <v>8000</v>
+      </c>
+      <c r="H11" s="260" t="n">
+        <v>7880</v>
+      </c>
+      <c r="I11" s="260" t="n">
+        <v>120</v>
+      </c>
+      <c r="J11" s="261">
+        <f>IFERROR(I11/(H11+I11),"")</f>
+        <v/>
+      </c>
+      <c r="K11" s="259" t="n"/>
+      <c r="L11" s="259" t="n"/>
+      <c r="M11" s="259" t="n"/>
+      <c r="N11" s="259" t="n"/>
+      <c r="O11" s="259" t="n"/>
+      <c r="P11" s="259" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q11" s="259" t="n"/>
+      <c r="R11" s="259" t="n"/>
+      <c r="S11" s="259" t="n"/>
     </row>
     <row r="12" hidden="1" ht="15" customHeight="1" s="246">
-      <c r="A12" s="193" t="n"/>
-      <c r="B12" s="194" t="n"/>
-      <c r="C12" s="194" t="n"/>
-      <c r="D12" s="194" t="n"/>
-      <c r="E12" s="194" t="n"/>
-      <c r="F12" s="194" t="n"/>
-      <c r="G12" s="195" t="n"/>
-      <c r="H12" s="195" t="n"/>
-      <c r="I12" s="195" t="n"/>
-      <c r="J12" s="196" t="n"/>
-      <c r="K12" s="194" t="n"/>
-      <c r="L12" s="194" t="n"/>
-      <c r="M12" s="194" t="n"/>
-      <c r="N12" s="194" t="n"/>
-      <c r="O12" s="194" t="n"/>
-      <c r="P12" s="194" t="n"/>
-      <c r="Q12" s="194" t="n"/>
-      <c r="R12" s="194" t="n"/>
-      <c r="S12" s="194" t="n"/>
+      <c r="A12" s="262" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B12" s="259" t="inlineStr">
+        <is>
+          <t>Lacquer-04</t>
+        </is>
+      </c>
+      <c r="C12" s="259" t="inlineStr">
+        <is>
+          <t>Golden Pearl Cosmetics (PVT) LTD</t>
+        </is>
+      </c>
+      <c r="D12" s="259" t="inlineStr">
+        <is>
+          <t>HELLO HAIR COLOR</t>
+        </is>
+      </c>
+      <c r="E12" s="259" t="n">
+        <v>30</v>
+      </c>
+      <c r="F12" s="259" t="n">
+        <v>6206</v>
+      </c>
+      <c r="G12" s="260" t="n">
+        <v>4000</v>
+      </c>
+      <c r="H12" s="260" t="n">
+        <v>3905</v>
+      </c>
+      <c r="I12" s="260" t="n">
+        <v>95</v>
+      </c>
+      <c r="J12" s="261">
+        <f>IFERROR(I12/(H12+I12),"")</f>
+        <v/>
+      </c>
+      <c r="K12" s="259" t="n"/>
+      <c r="L12" s="259" t="n"/>
+      <c r="M12" s="259" t="n"/>
+      <c r="N12" s="259" t="n"/>
+      <c r="O12" s="259" t="n"/>
+      <c r="P12" s="259" t="n"/>
+      <c r="Q12" s="259" t="n"/>
+      <c r="R12" s="259" t="n"/>
+      <c r="S12" s="259" t="n"/>
     </row>
     <row r="13" hidden="1" ht="15" customHeight="1" s="246">
-      <c r="A13" s="193" t="n"/>
-      <c r="B13" s="194" t="n"/>
-      <c r="C13" s="194" t="n"/>
-      <c r="D13" s="194" t="n"/>
-      <c r="E13" s="194" t="n"/>
-      <c r="F13" s="194" t="n"/>
-      <c r="G13" s="195" t="n"/>
-      <c r="H13" s="195" t="n"/>
-      <c r="I13" s="195" t="n"/>
-      <c r="J13" s="196" t="n"/>
-      <c r="K13" s="194" t="n"/>
-      <c r="L13" s="194" t="n"/>
-      <c r="M13" s="194" t="n"/>
-      <c r="N13" s="194" t="n"/>
-      <c r="O13" s="194" t="n"/>
-      <c r="P13" s="194" t="n"/>
-      <c r="Q13" s="194" t="n"/>
-      <c r="R13" s="194" t="n"/>
-      <c r="S13" s="194" t="n"/>
+      <c r="A13" s="262" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B13" s="259" t="inlineStr">
+        <is>
+          <t>Latex-01</t>
+        </is>
+      </c>
+      <c r="C13" s="259" t="inlineStr">
+        <is>
+          <t>Golden Pearl Cosmetics (PVT) LTD</t>
+        </is>
+      </c>
+      <c r="D13" s="259" t="inlineStr">
+        <is>
+          <t>HELLO HAIR COLOR</t>
+        </is>
+      </c>
+      <c r="E13" s="259" t="n">
+        <v>30</v>
+      </c>
+      <c r="F13" s="259" t="n">
+        <v>6206</v>
+      </c>
+      <c r="G13" s="260" t="n">
+        <v>22134</v>
+      </c>
+      <c r="H13" s="260" t="n">
+        <v>22124</v>
+      </c>
+      <c r="I13" s="260" t="n">
+        <v>10</v>
+      </c>
+      <c r="J13" s="261">
+        <f>IFERROR(I13/(H13+I13),"")</f>
+        <v/>
+      </c>
+      <c r="K13" s="259" t="n"/>
+      <c r="L13" s="259" t="n"/>
+      <c r="M13" s="259" t="n"/>
+      <c r="N13" s="259" t="n"/>
+      <c r="O13" s="259" t="n"/>
+      <c r="P13" s="259" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q13" s="259" t="n"/>
+      <c r="R13" s="259" t="n"/>
+      <c r="S13" s="259" t="n"/>
     </row>
     <row r="14" hidden="1" ht="15" customHeight="1" s="246">
-      <c r="A14" s="193" t="n"/>
-      <c r="B14" s="194" t="n"/>
-      <c r="C14" s="194" t="n"/>
-      <c r="D14" s="194" t="n"/>
-      <c r="E14" s="194" t="n"/>
-      <c r="F14" s="194" t="n"/>
-      <c r="G14" s="195" t="n"/>
-      <c r="H14" s="195" t="n"/>
-      <c r="I14" s="195" t="n"/>
-      <c r="J14" s="196" t="n"/>
-      <c r="K14" s="194" t="n"/>
-      <c r="L14" s="194" t="n"/>
-      <c r="M14" s="194" t="n"/>
-      <c r="N14" s="194" t="n"/>
-      <c r="O14" s="194" t="n"/>
-      <c r="P14" s="194" t="n"/>
-      <c r="Q14" s="194" t="n"/>
-      <c r="R14" s="194" t="n"/>
-      <c r="S14" s="194" t="n"/>
+      <c r="A14" s="262" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B14" s="259" t="inlineStr">
+        <is>
+          <t>PF Machine</t>
+        </is>
+      </c>
+      <c r="C14" s="259" t="inlineStr">
+        <is>
+          <t>Alpha Labs PVT LTD</t>
+        </is>
+      </c>
+      <c r="D14" s="259" t="inlineStr">
+        <is>
+          <t>TRANSPARENT BOTTLE 150ML</t>
+        </is>
+      </c>
+      <c r="E14" s="259" t="inlineStr">
+        <is>
+          <t>150 ml</t>
+        </is>
+      </c>
+      <c r="F14" s="259" t="n">
+        <v>8001</v>
+      </c>
+      <c r="G14" s="260" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="260" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="260" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="261">
+        <f>IFERROR(I14/(H14+I14),"")</f>
+        <v/>
+      </c>
+      <c r="K14" s="259" t="n"/>
+      <c r="L14" s="259" t="n"/>
+      <c r="M14" s="259" t="n"/>
+      <c r="N14" s="259" t="n"/>
+      <c r="O14" s="259" t="n">
+        <v>480</v>
+      </c>
+      <c r="P14" s="259" t="n"/>
+      <c r="Q14" s="259" t="n"/>
+      <c r="R14" s="259" t="n"/>
+      <c r="S14" s="259" t="n"/>
     </row>
     <row r="15" hidden="1" ht="15" customHeight="1" s="246">
-      <c r="A15" s="193" t="n"/>
-      <c r="B15" s="194" t="n"/>
-      <c r="C15" s="194" t="n"/>
-      <c r="D15" s="194" t="n"/>
-      <c r="E15" s="194" t="n"/>
-      <c r="F15" s="194" t="n"/>
-      <c r="G15" s="195" t="n"/>
-      <c r="H15" s="195" t="n"/>
-      <c r="I15" s="195" t="n"/>
-      <c r="J15" s="196" t="n"/>
-      <c r="K15" s="194" t="n"/>
-      <c r="L15" s="194" t="n"/>
-      <c r="M15" s="194" t="n"/>
-      <c r="N15" s="194" t="n"/>
-      <c r="O15" s="194" t="n"/>
-      <c r="P15" s="194" t="n"/>
-      <c r="Q15" s="194" t="n"/>
-      <c r="R15" s="194" t="n"/>
-      <c r="S15" s="194" t="n"/>
+      <c r="A15" s="262" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B15" s="259" t="inlineStr">
+        <is>
+          <t>Press-04</t>
+        </is>
+      </c>
+      <c r="C15" s="259" t="inlineStr">
+        <is>
+          <t>Mablay Beauty PVT LTD.</t>
+        </is>
+      </c>
+      <c r="D15" s="259" t="inlineStr">
+        <is>
+          <t>VINCE NURTURAL</t>
+        </is>
+      </c>
+      <c r="E15" s="259" t="n">
+        <v>30</v>
+      </c>
+      <c r="F15" s="259" t="n">
+        <v>5814</v>
+      </c>
+      <c r="G15" s="260" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="260" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="260" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="261">
+        <f>IFERROR(I15/(H15+I15),"")</f>
+        <v/>
+      </c>
+      <c r="K15" s="259" t="n"/>
+      <c r="L15" s="259" t="n"/>
+      <c r="M15" s="259" t="n"/>
+      <c r="N15" s="259" t="n"/>
+      <c r="O15" s="259" t="n"/>
+      <c r="P15" s="259" t="n"/>
+      <c r="Q15" s="259" t="n"/>
+      <c r="R15" s="259" t="n"/>
+      <c r="S15" s="259" t="n"/>
     </row>
     <row r="16" hidden="1" ht="15" customHeight="1" s="246">
-      <c r="A16" s="193" t="n"/>
-      <c r="B16" s="194" t="n"/>
-      <c r="C16" s="194" t="n"/>
-      <c r="D16" s="194" t="n"/>
-      <c r="E16" s="194" t="n"/>
-      <c r="F16" s="194" t="n"/>
-      <c r="G16" s="195" t="n"/>
-      <c r="H16" s="195" t="n"/>
-      <c r="I16" s="195" t="n"/>
-      <c r="J16" s="196" t="n"/>
-      <c r="K16" s="194" t="n"/>
-      <c r="L16" s="194" t="n"/>
-      <c r="M16" s="194" t="n"/>
-      <c r="N16" s="194" t="n"/>
-      <c r="O16" s="194" t="n"/>
-      <c r="P16" s="194" t="n"/>
-      <c r="Q16" s="194" t="n"/>
-      <c r="R16" s="194" t="n"/>
-      <c r="S16" s="194" t="n"/>
+      <c r="A16" s="262" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B16" s="259" t="inlineStr">
+        <is>
+          <t>Press-06</t>
+        </is>
+      </c>
+      <c r="C16" s="259" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D16" s="259" t="inlineStr">
+        <is>
+          <t>TUBES</t>
+        </is>
+      </c>
+      <c r="E16" s="259" t="n">
+        <v>25</v>
+      </c>
+      <c r="F16" s="259" t="n">
+        <v>3726</v>
+      </c>
+      <c r="G16" s="260" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H16" s="260" t="n">
+        <v>980</v>
+      </c>
+      <c r="I16" s="260" t="n">
+        <v>20</v>
+      </c>
+      <c r="J16" s="261">
+        <f>IFERROR(I16/(H16+I16),"")</f>
+        <v/>
+      </c>
+      <c r="K16" s="259" t="n"/>
+      <c r="L16" s="259" t="n"/>
+      <c r="M16" s="259" t="n"/>
+      <c r="N16" s="259" t="n"/>
+      <c r="O16" s="259" t="n"/>
+      <c r="P16" s="259" t="n"/>
+      <c r="Q16" s="259" t="n"/>
+      <c r="R16" s="259" t="n"/>
+      <c r="S16" s="259" t="n"/>
     </row>
     <row r="17" hidden="1" ht="15" customHeight="1" s="246">
-      <c r="A17" s="193" t="n"/>
-      <c r="B17" s="194" t="n"/>
-      <c r="C17" s="194" t="n"/>
-      <c r="D17" s="194" t="n"/>
-      <c r="E17" s="194" t="n"/>
-      <c r="F17" s="194" t="n"/>
-      <c r="G17" s="195" t="n"/>
-      <c r="H17" s="195" t="n"/>
-      <c r="I17" s="195" t="n"/>
-      <c r="J17" s="196" t="n"/>
-      <c r="K17" s="194" t="n"/>
-      <c r="L17" s="194" t="n"/>
-      <c r="M17" s="194" t="n"/>
-      <c r="N17" s="194" t="n"/>
-      <c r="O17" s="194" t="n"/>
-      <c r="P17" s="194" t="n"/>
-      <c r="Q17" s="194" t="n"/>
-      <c r="R17" s="194" t="n"/>
-      <c r="S17" s="194" t="n"/>
+      <c r="A17" s="262" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B17" s="259" t="inlineStr">
+        <is>
+          <t>Printing-03</t>
+        </is>
+      </c>
+      <c r="C17" s="259" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D17" s="259" t="inlineStr">
+        <is>
+          <t>TUBES</t>
+        </is>
+      </c>
+      <c r="E17" s="259" t="n">
+        <v>25</v>
+      </c>
+      <c r="F17" s="259" t="n">
+        <v>3726</v>
+      </c>
+      <c r="G17" s="260" t="n">
+        <v>12687</v>
+      </c>
+      <c r="H17" s="260" t="n">
+        <v>12432</v>
+      </c>
+      <c r="I17" s="260" t="n">
+        <v>255</v>
+      </c>
+      <c r="J17" s="261">
+        <f>IFERROR(I17/(H17+I17),"")</f>
+        <v/>
+      </c>
+      <c r="K17" s="259" t="n"/>
+      <c r="L17" s="259" t="n"/>
+      <c r="M17" s="259" t="n"/>
+      <c r="N17" s="259" t="n"/>
+      <c r="O17" s="259" t="n"/>
+      <c r="P17" s="259" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q17" s="259" t="n"/>
+      <c r="R17" s="259" t="n"/>
+      <c r="S17" s="259" t="n"/>
     </row>
     <row r="18" hidden="1" ht="15" customHeight="1" s="246">
-      <c r="A18" s="193" t="n"/>
-      <c r="B18" s="194" t="n"/>
-      <c r="C18" s="194" t="n"/>
-      <c r="D18" s="194" t="n"/>
-      <c r="E18" s="194" t="n"/>
-      <c r="F18" s="194" t="n"/>
-      <c r="G18" s="195" t="n"/>
-      <c r="H18" s="195" t="n"/>
-      <c r="I18" s="195" t="n"/>
-      <c r="J18" s="196" t="n"/>
-      <c r="K18" s="194" t="n"/>
-      <c r="L18" s="194" t="n"/>
-      <c r="M18" s="194" t="n"/>
-      <c r="N18" s="194" t="n"/>
-      <c r="O18" s="194" t="n"/>
-      <c r="P18" s="194" t="n"/>
-      <c r="Q18" s="194" t="n"/>
-      <c r="R18" s="194" t="n"/>
-      <c r="S18" s="194" t="n"/>
+      <c r="A18" s="262" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B18" s="259" t="inlineStr">
+        <is>
+          <t>Printing-04</t>
+        </is>
+      </c>
+      <c r="C18" s="259" t="inlineStr">
+        <is>
+          <t>Golden Pearl Cosmetics (PVT) LTD</t>
+        </is>
+      </c>
+      <c r="D18" s="259" t="inlineStr">
+        <is>
+          <t>HELLO HAIR COLOR</t>
+        </is>
+      </c>
+      <c r="E18" s="259" t="n">
+        <v>30</v>
+      </c>
+      <c r="F18" s="259" t="n">
+        <v>6206</v>
+      </c>
+      <c r="G18" s="260" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="260" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="260" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="261">
+        <f>IFERROR(I18/(H18+I18),"")</f>
+        <v/>
+      </c>
+      <c r="K18" s="259" t="n"/>
+      <c r="L18" s="259" t="n"/>
+      <c r="M18" s="259" t="n"/>
+      <c r="N18" s="259" t="n"/>
+      <c r="O18" s="259" t="n"/>
+      <c r="P18" s="259" t="n"/>
+      <c r="Q18" s="259" t="n"/>
+      <c r="R18" s="259" t="n"/>
+      <c r="S18" s="259" t="n"/>
     </row>
     <row r="19" hidden="1" ht="15" customHeight="1" s="246">
       <c r="A19" s="193" t="n"/>
@@ -49093,7 +49337,7 @@
     <row r="1" ht="30" customHeight="1" s="246">
       <c r="A1" s="253" t="inlineStr">
         <is>
-          <t>FG STOCK IN HAND — Last Updated: 02-Jun-2026</t>
+          <t>FG STOCK IN HAND — Last Updated: 03-Jun-2026</t>
         </is>
       </c>
     </row>
@@ -49152,31 +49396,31 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="246">
-      <c r="A4" s="289" t="n">
+      <c r="A4" s="295" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="289" t="n">
+      <c r="B4" s="295" t="n">
         <v>8001</v>
       </c>
-      <c r="C4" s="290" t="inlineStr">
+      <c r="C4" s="296" t="inlineStr">
         <is>
           <t>Alpha Labs PVT LTD</t>
         </is>
       </c>
-      <c r="D4" s="290" t="inlineStr">
+      <c r="D4" s="296" t="inlineStr">
         <is>
           <t>TRANSPARENT BOTTLE 150ML</t>
         </is>
       </c>
-      <c r="E4" s="289" t="inlineStr">
+      <c r="E4" s="295" t="inlineStr">
         <is>
           <t>150ml</t>
         </is>
       </c>
-      <c r="F4" s="291" t="n">
+      <c r="F4" s="297" t="n">
         <v>33465</v>
       </c>
-      <c r="G4" s="289" t="inlineStr">
+      <c r="G4" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -49192,38 +49436,38 @@
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="246">
-      <c r="A5" s="289" t="n">
+      <c r="A5" s="295" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="289" t="n">
+      <c r="B5" s="295" t="n">
         <v>3726</v>
       </c>
-      <c r="C5" s="290" t="inlineStr">
+      <c r="C5" s="296" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D5" s="290" t="inlineStr">
+      <c r="D5" s="296" t="inlineStr">
         <is>
           <t>TUBES</t>
         </is>
       </c>
-      <c r="E5" s="289" t="inlineStr">
+      <c r="E5" s="295" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="F5" s="291" t="n">
+      <c r="F5" s="297" t="n">
         <v>22512</v>
       </c>
-      <c r="G5" s="289" t="inlineStr">
+      <c r="G5" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
       <c r="H5" s="266" t="inlineStr">
         <is>
-          <t>Ready for dispatch</t>
+          <t>No JOF</t>
         </is>
       </c>
       <c r="I5" s="109">
@@ -49232,38 +49476,38 @@
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="246">
-      <c r="A6" s="289" t="n">
+      <c r="A6" s="295" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="289" t="n">
+      <c r="B6" s="295" t="n">
         <v>3447</v>
       </c>
-      <c r="C6" s="290" t="inlineStr">
+      <c r="C6" s="296" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D6" s="290" t="inlineStr">
+      <c r="D6" s="296" t="inlineStr">
         <is>
           <t>S 43 25MM</t>
         </is>
       </c>
-      <c r="E6" s="289" t="inlineStr">
+      <c r="E6" s="295" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="F6" s="291" t="n">
+      <c r="F6" s="297" t="n">
         <v>89000</v>
       </c>
-      <c r="G6" s="289" t="inlineStr">
+      <c r="G6" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
       <c r="H6" s="266" t="inlineStr">
         <is>
-          <t>Ready for dispatch</t>
+          <t>No JOF</t>
         </is>
       </c>
       <c r="I6" s="109">
@@ -49272,31 +49516,31 @@
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="246">
-      <c r="A7" s="289" t="n">
+      <c r="A7" s="295" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="289" t="n">
+      <c r="B7" s="295" t="n">
         <v>4050</v>
       </c>
-      <c r="C7" s="290" t="inlineStr">
+      <c r="C7" s="296" t="inlineStr">
         <is>
           <t>Professional Beauty Solution (PVT) LTD.Pakistan</t>
         </is>
       </c>
-      <c r="D7" s="290" t="inlineStr">
+      <c r="D7" s="296" t="inlineStr">
         <is>
           <t>EAZICOLOR PREMIUM HAIR COLOUR 60ML</t>
         </is>
       </c>
-      <c r="E7" s="289" t="inlineStr">
+      <c r="E7" s="295" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F7" s="291" t="n">
+      <c r="F7" s="297" t="n">
         <v>9450</v>
       </c>
-      <c r="G7" s="289" t="inlineStr">
+      <c r="G7" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -49312,31 +49556,31 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="246">
-      <c r="A8" s="289" t="n">
+      <c r="A8" s="295" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="289" t="n">
+      <c r="B8" s="295" t="n">
         <v>6337</v>
       </c>
-      <c r="C8" s="290" t="inlineStr">
+      <c r="C8" s="296" t="inlineStr">
         <is>
           <t>Al-Rehman Group</t>
         </is>
       </c>
-      <c r="D8" s="290" t="inlineStr">
+      <c r="D8" s="296" t="inlineStr">
         <is>
           <t>ACTIVE PRO HAIR COLOR CREAM 60ML</t>
         </is>
       </c>
-      <c r="E8" s="289" t="inlineStr">
+      <c r="E8" s="295" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F8" s="291" t="n">
+      <c r="F8" s="297" t="n">
         <v>15680</v>
       </c>
-      <c r="G8" s="289" t="inlineStr">
+      <c r="G8" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -49352,31 +49596,31 @@
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="246">
-      <c r="A9" s="289" t="n">
+      <c r="A9" s="295" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="289" t="n">
+      <c r="B9" s="295" t="n">
         <v>6416</v>
       </c>
-      <c r="C9" s="290" t="inlineStr">
+      <c r="C9" s="296" t="inlineStr">
         <is>
           <t>Al-Rehman Group</t>
         </is>
       </c>
-      <c r="D9" s="290" t="inlineStr">
+      <c r="D9" s="296" t="inlineStr">
         <is>
           <t>SIGNATURE HAIR COLOR CREAM 60ML</t>
         </is>
       </c>
-      <c r="E9" s="289" t="inlineStr">
+      <c r="E9" s="295" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="F9" s="291" t="n">
+      <c r="F9" s="297" t="n">
         <v>15435</v>
       </c>
-      <c r="G9" s="289" t="inlineStr">
+      <c r="G9" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -49392,31 +49636,31 @@
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="246">
-      <c r="A10" s="289" t="n">
+      <c r="A10" s="295" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="289" t="n">
+      <c r="B10" s="295" t="n">
         <v>5782</v>
       </c>
-      <c r="C10" s="290" t="inlineStr">
+      <c r="C10" s="296" t="inlineStr">
         <is>
           <t>Mega Grey</t>
         </is>
       </c>
-      <c r="D10" s="290" t="inlineStr">
+      <c r="D10" s="296" t="inlineStr">
         <is>
           <t>M.G</t>
         </is>
       </c>
-      <c r="E10" s="289" t="inlineStr">
+      <c r="E10" s="295" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="F10" s="291" t="n">
+      <c r="F10" s="297" t="n">
         <v>63648</v>
       </c>
-      <c r="G10" s="289" t="inlineStr">
+      <c r="G10" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -49432,31 +49676,31 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="246">
-      <c r="A11" s="289" t="n">
+      <c r="A11" s="295" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="289" t="n">
+      <c r="B11" s="295" t="n">
         <v>6531</v>
       </c>
-      <c r="C11" s="290" t="inlineStr">
+      <c r="C11" s="296" t="inlineStr">
         <is>
           <t>Adore</t>
         </is>
       </c>
-      <c r="D11" s="290" t="inlineStr">
+      <c r="D11" s="296" t="inlineStr">
         <is>
           <t>V-HC BLACK</t>
         </is>
       </c>
-      <c r="E11" s="289" t="inlineStr">
+      <c r="E11" s="295" t="inlineStr">
         <is>
           <t>35</t>
         </is>
       </c>
-      <c r="F11" s="291" t="n">
+      <c r="F11" s="297" t="n">
         <v>4380</v>
       </c>
-      <c r="G11" s="289" t="inlineStr">
+      <c r="G11" s="295" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -49472,38 +49716,38 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="246">
-      <c r="A12" s="292" t="n">
+      <c r="A12" s="295" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="292" t="n">
-        <v>6515</v>
-      </c>
-      <c r="C12" s="293" t="inlineStr">
-        <is>
-          <t>Samsol International Private Limited</t>
-        </is>
-      </c>
-      <c r="D12" s="293" t="inlineStr">
-        <is>
-          <t>H.H 100GM</t>
-        </is>
-      </c>
-      <c r="E12" s="292" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="F12" s="294" t="n">
-        <v>38896</v>
-      </c>
-      <c r="G12" s="292" t="inlineStr">
-        <is>
-          <t>Not Ready</t>
-        </is>
-      </c>
-      <c r="H12" s="270" t="inlineStr">
-        <is>
-          <t>To be dispatch after packing</t>
+      <c r="B12" s="295" t="n">
+        <v>6206</v>
+      </c>
+      <c r="C12" s="296" t="inlineStr">
+        <is>
+          <t>Golden Pearl Cosmetics (PVT) LTD</t>
+        </is>
+      </c>
+      <c r="D12" s="296" t="inlineStr">
+        <is>
+          <t>HELLO HAIR COLOR</t>
+        </is>
+      </c>
+      <c r="E12" s="295" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="F12" s="297" t="n">
+        <v>35000</v>
+      </c>
+      <c r="G12" s="295" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="H12" s="266" t="inlineStr">
+        <is>
+          <t>No JOF</t>
         </is>
       </c>
       <c r="I12" s="109">
@@ -49512,31 +49756,31 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="246">
-      <c r="A13" s="292" t="n">
+      <c r="A13" s="298" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="292" t="n">
-        <v>6530</v>
-      </c>
-      <c r="C13" s="293" t="inlineStr">
-        <is>
-          <t>Adore</t>
-        </is>
-      </c>
-      <c r="D13" s="293" t="inlineStr">
-        <is>
-          <t>V- HC BROWN</t>
-        </is>
-      </c>
-      <c r="E13" s="292" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="F13" s="294" t="n">
-        <v>15000</v>
-      </c>
-      <c r="G13" s="292" t="inlineStr">
+      <c r="B13" s="298" t="n">
+        <v>6515</v>
+      </c>
+      <c r="C13" s="299" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D13" s="299" t="inlineStr">
+        <is>
+          <t>H.H 100GM</t>
+        </is>
+      </c>
+      <c r="E13" s="298" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="F13" s="300" t="n">
+        <v>38896</v>
+      </c>
+      <c r="G13" s="298" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -49552,31 +49796,31 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="246">
-      <c r="A14" s="292" t="n">
+      <c r="A14" s="298" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="292" t="n">
-        <v>6206</v>
-      </c>
-      <c r="C14" s="293" t="inlineStr">
-        <is>
-          <t>Golden Pearl Cosmetics (PVT) LTD</t>
-        </is>
-      </c>
-      <c r="D14" s="293" t="inlineStr">
-        <is>
-          <t>HELLO HAIR COLOR</t>
-        </is>
-      </c>
-      <c r="E14" s="292" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="F14" s="294" t="n">
-        <v>98674</v>
-      </c>
-      <c r="G14" s="292" t="inlineStr">
+      <c r="B14" s="298" t="n">
+        <v>6530</v>
+      </c>
+      <c r="C14" s="299" t="inlineStr">
+        <is>
+          <t>Adore</t>
+        </is>
+      </c>
+      <c r="D14" s="299" t="inlineStr">
+        <is>
+          <t>V- HC BROWN</t>
+        </is>
+      </c>
+      <c r="E14" s="298" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="F14" s="300" t="n">
+        <v>15000</v>
+      </c>
+      <c r="G14" s="298" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -49592,31 +49836,31 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="246">
-      <c r="A15" s="292" t="n">
+      <c r="A15" s="298" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="292" t="n">
-        <v>3726</v>
-      </c>
-      <c r="C15" s="293" t="inlineStr">
-        <is>
-          <t>Samsol International Private Limited</t>
-        </is>
-      </c>
-      <c r="D15" s="293" t="inlineStr">
-        <is>
-          <t>TUBES</t>
-        </is>
-      </c>
-      <c r="E15" s="292" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="F15" s="294" t="n">
-        <v>9744</v>
-      </c>
-      <c r="G15" s="292" t="inlineStr">
+      <c r="B15" s="298" t="n">
+        <v>6206</v>
+      </c>
+      <c r="C15" s="299" t="inlineStr">
+        <is>
+          <t>Golden Pearl Cosmetics (PVT) LTD</t>
+        </is>
+      </c>
+      <c r="D15" s="299" t="inlineStr">
+        <is>
+          <t>HELLO HAIR COLOR</t>
+        </is>
+      </c>
+      <c r="E15" s="298" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="F15" s="300" t="n">
+        <v>63674</v>
+      </c>
+      <c r="G15" s="298" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -49632,38 +49876,38 @@
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="246">
-      <c r="A16" s="292" t="n">
+      <c r="A16" s="298" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="292" t="n">
-        <v>5782</v>
-      </c>
-      <c r="C16" s="293" t="inlineStr">
-        <is>
-          <t>Mega Grey</t>
-        </is>
-      </c>
-      <c r="D16" s="293" t="inlineStr">
-        <is>
-          <t>M.G</t>
-        </is>
-      </c>
-      <c r="E16" s="292" t="inlineStr">
-        <is>
-          <t>32</t>
-        </is>
-      </c>
-      <c r="F16" s="294" t="n">
-        <v>10500</v>
-      </c>
-      <c r="G16" s="292" t="inlineStr">
+      <c r="B16" s="298" t="n">
+        <v>3726</v>
+      </c>
+      <c r="C16" s="299" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D16" s="299" t="inlineStr">
+        <is>
+          <t>TUBES</t>
+        </is>
+      </c>
+      <c r="E16" s="298" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="F16" s="300" t="n">
+        <v>22176</v>
+      </c>
+      <c r="G16" s="298" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
       </c>
       <c r="H16" s="270" t="inlineStr">
         <is>
-          <t>Cap Not Available</t>
+          <t>To be dispatch after packing</t>
         </is>
       </c>
       <c r="I16" s="110">
@@ -49672,31 +49916,31 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="246">
-      <c r="A17" s="292" t="n">
+      <c r="A17" s="298" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="292" t="n">
-        <v>6624</v>
-      </c>
-      <c r="C17" s="293" t="inlineStr">
-        <is>
-          <t>Samsol International Private Limited</t>
-        </is>
-      </c>
-      <c r="D17" s="293" t="inlineStr">
-        <is>
-          <t>S-45 DIA 19MM</t>
-        </is>
-      </c>
-      <c r="E17" s="292" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="F17" s="294" t="n">
-        <v>15288</v>
-      </c>
-      <c r="G17" s="292" t="inlineStr">
+      <c r="B17" s="298" t="n">
+        <v>5782</v>
+      </c>
+      <c r="C17" s="299" t="inlineStr">
+        <is>
+          <t>Mega Grey</t>
+        </is>
+      </c>
+      <c r="D17" s="299" t="inlineStr">
+        <is>
+          <t>M.G</t>
+        </is>
+      </c>
+      <c r="E17" s="298" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="F17" s="300" t="n">
+        <v>10500</v>
+      </c>
+      <c r="G17" s="298" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -49712,31 +49956,31 @@
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="246">
-      <c r="A18" s="292" t="n">
+      <c r="A18" s="298" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="292" t="n">
-        <v>5699</v>
-      </c>
-      <c r="C18" s="293" t="inlineStr">
+      <c r="B18" s="298" t="n">
+        <v>6624</v>
+      </c>
+      <c r="C18" s="299" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D18" s="293" t="inlineStr">
-        <is>
-          <t>S-43 DIA 20.5</t>
-        </is>
-      </c>
-      <c r="E18" s="292" t="inlineStr">
-        <is>
-          <t>20.5</t>
-        </is>
-      </c>
-      <c r="F18" s="294" t="n">
-        <v>13770</v>
-      </c>
-      <c r="G18" s="292" t="inlineStr">
+      <c r="D18" s="299" t="inlineStr">
+        <is>
+          <t>S-45 DIA 19MM</t>
+        </is>
+      </c>
+      <c r="E18" s="298" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="F18" s="300" t="n">
+        <v>15288</v>
+      </c>
+      <c r="G18" s="298" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
@@ -49752,38 +49996,38 @@
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="246">
-      <c r="A19" s="292" t="n">
+      <c r="A19" s="298" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="292" t="n">
-        <v>5731</v>
-      </c>
-      <c r="C19" s="293" t="inlineStr">
+      <c r="B19" s="298" t="n">
+        <v>5699</v>
+      </c>
+      <c r="C19" s="299" t="inlineStr">
         <is>
           <t>Samsol International Private Limited</t>
         </is>
       </c>
-      <c r="D19" s="293" t="inlineStr">
-        <is>
-          <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
-        </is>
-      </c>
-      <c r="E19" s="292" t="inlineStr">
+      <c r="D19" s="299" t="inlineStr">
+        <is>
+          <t>S-43 DIA 20.5</t>
+        </is>
+      </c>
+      <c r="E19" s="298" t="inlineStr">
         <is>
           <t>20.5</t>
         </is>
       </c>
-      <c r="F19" s="294" t="n">
-        <v>51000</v>
-      </c>
-      <c r="G19" s="292" t="inlineStr">
+      <c r="F19" s="300" t="n">
+        <v>13770</v>
+      </c>
+      <c r="G19" s="298" t="inlineStr">
         <is>
           <t>Not Ready</t>
         </is>
       </c>
       <c r="H19" s="270" t="inlineStr">
         <is>
-          <t>Cap Not Available</t>
+          <t>To be dispatch after packing</t>
         </is>
       </c>
       <c r="I19" s="110">
@@ -49792,28 +50036,80 @@
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="246">
-      <c r="A20" s="271" t="n"/>
-      <c r="B20" s="271" t="n"/>
-      <c r="C20" s="272" t="n"/>
-      <c r="D20" s="272" t="n"/>
-      <c r="E20" s="271" t="n"/>
-      <c r="F20" s="273" t="n"/>
-      <c r="G20" s="271" t="n"/>
-      <c r="H20" s="274" t="n"/>
+      <c r="A20" s="298" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="298" t="n">
+        <v>5731</v>
+      </c>
+      <c r="C20" s="299" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D20" s="299" t="inlineStr">
+        <is>
+          <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
+        </is>
+      </c>
+      <c r="E20" s="298" t="inlineStr">
+        <is>
+          <t>20.5</t>
+        </is>
+      </c>
+      <c r="F20" s="300" t="n">
+        <v>13260</v>
+      </c>
+      <c r="G20" s="298" t="inlineStr">
+        <is>
+          <t>Not Ready</t>
+        </is>
+      </c>
+      <c r="H20" s="270" t="inlineStr">
+        <is>
+          <t>To be dispatch after packing</t>
+        </is>
+      </c>
       <c r="I20" s="110">
         <f>IFERROR(SUMPRODUCT((TableBOM[Product ID]=B20)*(TableBOM[Material Category]="CAP")*TableBOM[Item ID]),0)</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="246">
-      <c r="A21" s="271" t="n"/>
-      <c r="B21" s="271" t="n"/>
-      <c r="C21" s="272" t="n"/>
-      <c r="D21" s="272" t="n"/>
-      <c r="E21" s="271" t="n"/>
-      <c r="F21" s="273" t="n"/>
-      <c r="G21" s="271" t="n"/>
-      <c r="H21" s="274" t="n"/>
+      <c r="A21" s="298" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="298" t="n">
+        <v>5731</v>
+      </c>
+      <c r="C21" s="299" t="inlineStr">
+        <is>
+          <t>Samsol International Private Limited</t>
+        </is>
+      </c>
+      <c r="D21" s="299" t="inlineStr">
+        <is>
+          <t>SAMSOL HAIR COLOR 45 DIA 20.5 MM</t>
+        </is>
+      </c>
+      <c r="E21" s="298" t="inlineStr">
+        <is>
+          <t>20.5</t>
+        </is>
+      </c>
+      <c r="F21" s="300" t="n">
+        <v>37740</v>
+      </c>
+      <c r="G21" s="298" t="inlineStr">
+        <is>
+          <t>Not Ready</t>
+        </is>
+      </c>
+      <c r="H21" s="270" t="inlineStr">
+        <is>
+          <t>Cap Not Available</t>
+        </is>
+      </c>
       <c r="I21" s="110">
         <f>IFERROR(SUMPRODUCT((TableBOM[Product ID]=B21)*(TableBOM[Material Category]="CAP")*TableBOM[Item ID]),0)</f>
         <v/>

</xml_diff>